<commit_message>
Fixed one store that had poor data (variedades)
</commit_message>
<xml_diff>
--- a/data/stores/agmarkets_bronx_cd2_snap_eligibility_edited.xlsx
+++ b/data/stores/agmarkets_bronx_cd2_snap_eligibility_edited.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samia\Code_Projects\grocery_subsidy_analysis\data\stores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED1AA222-3274-4AE0-8761-06E86A39C9A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2930B08B-E220-4C70-A8EF-A7393C593453}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="13152" windowHeight="11112" xr2:uid="{9D3F1190-A07F-4A30-BD0A-96434696D40A}"/>
+    <workbookView xWindow="1464" yWindow="1464" windowWidth="17280" windowHeight="8880" xr2:uid="{9D3F1190-A07F-4A30-BD0A-96434696D40A}"/>
   </bookViews>
   <sheets>
     <sheet name="agmarkets_bronx_cd2_snap_eligib" sheetId="1" r:id="rId1"/>
@@ -7063,7 +7063,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B96B7A09-E894-4653-AE09-295EC567A304}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:AC138"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -7169,7 +7168,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -7246,7 +7245,7 @@
         <v>45473</v>
       </c>
     </row>
-    <row r="3" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>27</v>
       </c>
@@ -7323,7 +7322,7 @@
         <v>44609</v>
       </c>
     </row>
-    <row r="4" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -7400,7 +7399,7 @@
         <v>45798</v>
       </c>
     </row>
-    <row r="5" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -7462,7 +7461,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -7539,7 +7538,7 @@
         <v>45896</v>
       </c>
     </row>
-    <row r="7" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>27</v>
       </c>
@@ -7613,7 +7612,7 @@
         <v>45520</v>
       </c>
     </row>
-    <row r="8" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>27</v>
       </c>
@@ -7690,7 +7689,7 @@
         <v>45775</v>
       </c>
     </row>
-    <row r="9" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>27</v>
       </c>
@@ -7767,7 +7766,7 @@
         <v>44616</v>
       </c>
     </row>
-    <row r="10" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -7844,7 +7843,7 @@
         <v>45742</v>
       </c>
     </row>
-    <row r="11" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>27</v>
       </c>
@@ -7921,7 +7920,7 @@
         <v>45533</v>
       </c>
     </row>
-    <row r="12" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>27</v>
       </c>
@@ -8001,7 +8000,7 @@
         <v>40924</v>
       </c>
     </row>
-    <row r="13" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>27</v>
       </c>
@@ -8075,7 +8074,7 @@
         <v>42993</v>
       </c>
     </row>
-    <row r="14" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>27</v>
       </c>
@@ -8152,7 +8151,7 @@
         <v>45614</v>
       </c>
     </row>
-    <row r="15" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -8226,7 +8225,7 @@
         <v>45530</v>
       </c>
     </row>
-    <row r="16" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>27</v>
       </c>
@@ -8303,7 +8302,7 @@
         <v>45491</v>
       </c>
     </row>
-    <row r="17" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>27</v>
       </c>
@@ -8377,7 +8376,7 @@
         <v>45511</v>
       </c>
     </row>
-    <row r="18" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>27</v>
       </c>
@@ -8454,7 +8453,7 @@
         <v>45106</v>
       </c>
     </row>
-    <row r="19" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>27</v>
       </c>
@@ -8528,7 +8527,7 @@
         <v>45551</v>
       </c>
     </row>
-    <row r="20" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>27</v>
       </c>
@@ -8602,7 +8601,7 @@
         <v>45525</v>
       </c>
     </row>
-    <row r="21" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>27</v>
       </c>
@@ -8676,7 +8675,7 @@
         <v>45638</v>
       </c>
     </row>
-    <row r="22" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>27</v>
       </c>
@@ -8753,7 +8752,7 @@
         <v>45118</v>
       </c>
     </row>
-    <row r="23" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>27</v>
       </c>
@@ -8827,7 +8826,7 @@
         <v>45531</v>
       </c>
     </row>
-    <row r="24" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>27</v>
       </c>
@@ -8901,7 +8900,7 @@
         <v>45008</v>
       </c>
     </row>
-    <row r="25" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>27</v>
       </c>
@@ -8978,7 +8977,7 @@
         <v>45537</v>
       </c>
     </row>
-    <row r="26" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>27</v>
       </c>
@@ -9040,7 +9039,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="27" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>27</v>
       </c>
@@ -9117,7 +9116,7 @@
         <v>45259</v>
       </c>
     </row>
-    <row r="28" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -9194,7 +9193,7 @@
         <v>45153</v>
       </c>
     </row>
-    <row r="29" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -9268,7 +9267,7 @@
         <v>44945</v>
       </c>
     </row>
-    <row r="30" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>27</v>
       </c>
@@ -9348,7 +9347,7 @@
         <v>45917</v>
       </c>
     </row>
-    <row r="31" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>27</v>
       </c>
@@ -9422,7 +9421,7 @@
         <v>44984</v>
       </c>
     </row>
-    <row r="32" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>27</v>
       </c>
@@ -9481,7 +9480,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="33" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>27</v>
       </c>
@@ -9558,7 +9557,7 @@
         <v>45975</v>
       </c>
     </row>
-    <row r="34" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>27</v>
       </c>
@@ -9632,7 +9631,7 @@
         <v>44770</v>
       </c>
     </row>
-    <row r="35" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>27</v>
       </c>
@@ -9709,7 +9708,7 @@
         <v>44739</v>
       </c>
     </row>
-    <row r="36" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>27</v>
       </c>
@@ -9783,7 +9782,7 @@
         <v>44725</v>
       </c>
     </row>
-    <row r="37" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>27</v>
       </c>
@@ -9860,7 +9859,7 @@
         <v>44806</v>
       </c>
     </row>
-    <row r="38" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>27</v>
       </c>
@@ -9940,7 +9939,7 @@
         <v>44018</v>
       </c>
     </row>
-    <row r="39" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>27</v>
       </c>
@@ -10014,7 +10013,7 @@
         <v>45259</v>
       </c>
     </row>
-    <row r="40" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>27</v>
       </c>
@@ -10091,7 +10090,7 @@
         <v>33015</v>
       </c>
     </row>
-    <row r="41" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>27</v>
       </c>
@@ -10168,7 +10167,7 @@
         <v>41729</v>
       </c>
     </row>
-    <row r="42" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>27</v>
       </c>
@@ -10230,7 +10229,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="43" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>27</v>
       </c>
@@ -10304,7 +10303,7 @@
         <v>44767</v>
       </c>
     </row>
-    <row r="44" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>27</v>
       </c>
@@ -10366,7 +10365,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="45" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>27</v>
       </c>
@@ -10443,7 +10442,7 @@
         <v>45064</v>
       </c>
     </row>
-    <row r="46" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>27</v>
       </c>
@@ -10517,7 +10516,7 @@
         <v>43956</v>
       </c>
     </row>
-    <row r="47" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>27</v>
       </c>
@@ -10597,7 +10596,7 @@
         <v>45614</v>
       </c>
     </row>
-    <row r="48" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>27</v>
       </c>
@@ -10671,7 +10670,7 @@
         <v>44587</v>
       </c>
     </row>
-    <row r="49" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>27</v>
       </c>
@@ -10751,7 +10750,7 @@
         <v>45889</v>
       </c>
     </row>
-    <row r="50" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>27</v>
       </c>
@@ -10813,7 +10812,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="51" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>27</v>
       </c>
@@ -10890,7 +10889,7 @@
         <v>44211</v>
       </c>
     </row>
-    <row r="52" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>27</v>
       </c>
@@ -10967,7 +10966,7 @@
         <v>44455</v>
       </c>
     </row>
-    <row r="53" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>27</v>
       </c>
@@ -11044,7 +11043,7 @@
         <v>44586</v>
       </c>
     </row>
-    <row r="54" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>27</v>
       </c>
@@ -11121,7 +11120,7 @@
         <v>45273</v>
       </c>
     </row>
-    <row r="55" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>27</v>
       </c>
@@ -11201,7 +11200,7 @@
         <v>45274</v>
       </c>
     </row>
-    <row r="56" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>27</v>
       </c>
@@ -11278,7 +11277,7 @@
         <v>43738</v>
       </c>
     </row>
-    <row r="57" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>27</v>
       </c>
@@ -11358,7 +11357,7 @@
         <v>40924</v>
       </c>
     </row>
-    <row r="58" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>27</v>
       </c>
@@ -11435,7 +11434,7 @@
         <v>43731</v>
       </c>
     </row>
-    <row r="59" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>27</v>
       </c>
@@ -11515,7 +11514,7 @@
         <v>43791</v>
       </c>
     </row>
-    <row r="60" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>27</v>
       </c>
@@ -11595,7 +11594,7 @@
         <v>45113</v>
       </c>
     </row>
-    <row r="61" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>27</v>
       </c>
@@ -11672,7 +11671,7 @@
         <v>45923</v>
       </c>
     </row>
-    <row r="62" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>27</v>
       </c>
@@ -11749,7 +11748,7 @@
         <v>44696</v>
       </c>
     </row>
-    <row r="63" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>27</v>
       </c>
@@ -11826,7 +11825,7 @@
         <v>42955</v>
       </c>
     </row>
-    <row r="64" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>27</v>
       </c>
@@ -11900,7 +11899,7 @@
         <v>44246</v>
       </c>
     </row>
-    <row r="65" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>27</v>
       </c>
@@ -11977,7 +11976,7 @@
         <v>45572</v>
       </c>
     </row>
-    <row r="66" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>27</v>
       </c>
@@ -12054,7 +12053,7 @@
         <v>45890</v>
       </c>
     </row>
-    <row r="67" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>27</v>
       </c>
@@ -12134,7 +12133,7 @@
         <v>43620</v>
       </c>
     </row>
-    <row r="68" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>27</v>
       </c>
@@ -12211,7 +12210,7 @@
         <v>45742</v>
       </c>
     </row>
-    <row r="69" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>27</v>
       </c>
@@ -12291,7 +12290,7 @@
         <v>45923</v>
       </c>
     </row>
-    <row r="70" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>27</v>
       </c>
@@ -12371,7 +12370,7 @@
         <v>41730</v>
       </c>
     </row>
-    <row r="71" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>27</v>
       </c>
@@ -12451,7 +12450,7 @@
         <v>44726</v>
       </c>
     </row>
-    <row r="72" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>27</v>
       </c>
@@ -12525,7 +12524,7 @@
         <v>45929</v>
       </c>
     </row>
-    <row r="73" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>27</v>
       </c>
@@ -12605,7 +12604,7 @@
         <v>45049</v>
       </c>
     </row>
-    <row r="74" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>27</v>
       </c>
@@ -12679,7 +12678,7 @@
         <v>45812</v>
       </c>
     </row>
-    <row r="75" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>27</v>
       </c>
@@ -12756,7 +12755,7 @@
         <v>42650</v>
       </c>
     </row>
-    <row r="76" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>27</v>
       </c>
@@ -12833,7 +12832,7 @@
         <v>45117</v>
       </c>
     </row>
-    <row r="77" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>27</v>
       </c>
@@ -12913,7 +12912,7 @@
         <v>45714</v>
       </c>
     </row>
-    <row r="78" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>27</v>
       </c>
@@ -12990,7 +12989,7 @@
         <v>42993</v>
       </c>
     </row>
-    <row r="79" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>27</v>
       </c>
@@ -13067,7 +13066,7 @@
         <v>45890</v>
       </c>
     </row>
-    <row r="80" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>27</v>
       </c>
@@ -13144,7 +13143,7 @@
         <v>45153</v>
       </c>
     </row>
-    <row r="81" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>27</v>
       </c>
@@ -13221,7 +13220,7 @@
         <v>43218</v>
       </c>
     </row>
-    <row r="82" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>27</v>
       </c>
@@ -13283,7 +13282,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="83" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>27</v>
       </c>
@@ -13357,7 +13356,7 @@
         <v>43706</v>
       </c>
     </row>
-    <row r="84" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>27</v>
       </c>
@@ -13434,7 +13433,7 @@
         <v>44727</v>
       </c>
     </row>
-    <row r="85" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>27</v>
       </c>
@@ -13508,7 +13507,7 @@
         <v>42993</v>
       </c>
     </row>
-    <row r="86" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>27</v>
       </c>
@@ -13585,7 +13584,7 @@
         <v>44120</v>
       </c>
     </row>
-    <row r="87" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>27</v>
       </c>
@@ -13665,7 +13664,7 @@
         <v>45972</v>
       </c>
     </row>
-    <row r="88" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>27</v>
       </c>
@@ -13739,7 +13738,7 @@
         <v>45761</v>
       </c>
     </row>
-    <row r="89" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>27</v>
       </c>
@@ -13830,7 +13829,7 @@
         <v>29</v>
       </c>
       <c r="F90">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G90" t="s">
         <v>69</v>
@@ -13890,7 +13889,7 @@
         <v>42460</v>
       </c>
     </row>
-    <row r="91" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>27</v>
       </c>
@@ -13967,7 +13966,7 @@
         <v>45796</v>
       </c>
     </row>
-    <row r="92" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>27</v>
       </c>
@@ -14121,7 +14120,7 @@
         <v>42782</v>
       </c>
     </row>
-    <row r="94" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>27</v>
       </c>
@@ -14183,7 +14182,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="95" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>27</v>
       </c>
@@ -14260,7 +14259,7 @@
         <v>42558</v>
       </c>
     </row>
-    <row r="96" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>27</v>
       </c>
@@ -14337,7 +14336,7 @@
         <v>43616</v>
       </c>
     </row>
-    <row r="97" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>27</v>
       </c>
@@ -14417,7 +14416,7 @@
         <v>43423</v>
       </c>
     </row>
-    <row r="98" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>27</v>
       </c>
@@ -14479,7 +14478,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="99" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>27</v>
       </c>
@@ -14553,7 +14552,7 @@
         <v>42366</v>
       </c>
     </row>
-    <row r="100" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>27</v>
       </c>
@@ -14627,7 +14626,7 @@
         <v>45839</v>
       </c>
     </row>
-    <row r="101" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>27</v>
       </c>
@@ -14704,7 +14703,7 @@
         <v>44357</v>
       </c>
     </row>
-    <row r="102" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>27</v>
       </c>
@@ -14781,7 +14780,7 @@
         <v>45223</v>
       </c>
     </row>
-    <row r="103" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>27</v>
       </c>
@@ -14843,7 +14842,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="104" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>27</v>
       </c>
@@ -14905,7 +14904,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="105" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>27</v>
       </c>
@@ -14982,7 +14981,7 @@
         <v>44806</v>
       </c>
     </row>
-    <row r="106" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>27</v>
       </c>
@@ -15062,7 +15061,7 @@
         <v>42940</v>
       </c>
     </row>
-    <row r="107" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>27</v>
       </c>
@@ -15139,7 +15138,7 @@
         <v>45530</v>
       </c>
     </row>
-    <row r="108" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>27</v>
       </c>
@@ -15201,7 +15200,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="109" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>27</v>
       </c>
@@ -15358,7 +15357,7 @@
         <v>42460</v>
       </c>
     </row>
-    <row r="111" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>27</v>
       </c>
@@ -15515,7 +15514,7 @@
         <v>37187</v>
       </c>
     </row>
-    <row r="113" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>27</v>
       </c>
@@ -15654,7 +15653,7 @@
         <v>35306</v>
       </c>
     </row>
-    <row r="115" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>27</v>
       </c>
@@ -15734,7 +15733,7 @@
         <v>45348</v>
       </c>
     </row>
-    <row r="116" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>27</v>
       </c>
@@ -15811,7 +15810,7 @@
         <v>40633</v>
       </c>
     </row>
-    <row r="117" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>27</v>
       </c>
@@ -15888,7 +15887,7 @@
         <v>40457</v>
       </c>
     </row>
-    <row r="118" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>27</v>
       </c>
@@ -15965,7 +15964,7 @@
         <v>44462</v>
       </c>
     </row>
-    <row r="119" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>27</v>
       </c>
@@ -16045,7 +16044,7 @@
         <v>45516</v>
       </c>
     </row>
-    <row r="120" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>27</v>
       </c>
@@ -16122,7 +16121,7 @@
         <v>45772</v>
       </c>
     </row>
-    <row r="121" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>27</v>
       </c>
@@ -16199,7 +16198,7 @@
         <v>45768</v>
       </c>
     </row>
-    <row r="122" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>27</v>
       </c>
@@ -16279,7 +16278,7 @@
         <v>42731</v>
       </c>
     </row>
-    <row r="123" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>27</v>
       </c>
@@ -16356,7 +16355,7 @@
         <v>44727</v>
       </c>
     </row>
-    <row r="124" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>27</v>
       </c>
@@ -16418,7 +16417,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="125" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>27</v>
       </c>
@@ -16495,7 +16494,7 @@
         <v>45834</v>
       </c>
     </row>
-    <row r="126" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>27</v>
       </c>
@@ -16572,7 +16571,7 @@
         <v>42558</v>
       </c>
     </row>
-    <row r="127" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>27</v>
       </c>
@@ -16649,7 +16648,7 @@
         <v>38912</v>
       </c>
     </row>
-    <row r="128" spans="1:29" hidden="1" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>27</v>
       </c>
@@ -16883,7 +16882,7 @@
         <v>44351</v>
       </c>
     </row>
-    <row r="131" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>27</v>
       </c>
@@ -16960,7 +16959,7 @@
         <v>41487</v>
       </c>
     </row>
-    <row r="132" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>27</v>
       </c>
@@ -17191,7 +17190,7 @@
         <v>30740</v>
       </c>
     </row>
-    <row r="135" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>27</v>
       </c>
@@ -17268,7 +17267,7 @@
         <v>45637</v>
       </c>
     </row>
-    <row r="136" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>27</v>
       </c>
@@ -17422,7 +17421,7 @@
         <v>38371</v>
       </c>
     </row>
-    <row r="138" spans="1:28" hidden="1" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>27</v>
       </c>
@@ -17500,13 +17499,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC138" xr:uid="{B96B7A09-E894-4653-AE09-295EC567A304}">
-    <filterColumn colId="5">
-      <filters>
-        <filter val="1"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:AC138" xr:uid="{B96B7A09-E894-4653-AE09-295EC567A304}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>